<commit_message>
create class to calculate mixture average compositions
</commit_message>
<xml_diff>
--- a/UnifacDortmund/Experimental_Data/data/profile_coeffs.xlsx
+++ b/UnifacDortmund/Experimental_Data/data/profile_coeffs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Juan\proyectos_personales\Maestría\Materias\Tesis\oleosim\UnifacDortmund\Experimental_Data\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD8A0F0B-2D4C-4148-87CB-59A8A4787BC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{030E3B24-7CCE-4E96-AB03-4BB4BCDD9221}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -156,7 +156,7 @@
       <numFmt numFmtId="165" formatCode="#,##0.000;[Red]\-#,##0.000"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="165" formatCode="#,##0.000;[Red]\-#,##0.000"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="165" formatCode="#,##0.000;[Red]\-#,##0.000"/>
@@ -165,7 +165,7 @@
       <numFmt numFmtId="165" formatCode="#,##0.000;[Red]\-#,##0.000"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="#,##0.000;[Red]\-#,##0.000"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="#,##0;[Red]\-#,##0"/>
@@ -192,10 +192,10 @@
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="MAG/DAG Profile?"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Additional FAME Profile?"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Acid mix Profile?"/>
-    <tableColumn id="9" xr3:uid="{9F057E55-9F2C-4F9F-BF85-42F7D5BDEAEE}" name="Type Alcohol" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="m" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="n" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="p" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{9F057E55-9F2C-4F9F-BF85-42F7D5BDEAEE}" name="Type Alcohol" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="m" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="n" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="p" dataDxfId="1"/>
     <tableColumn id="10" xr3:uid="{A79D96DD-C468-4203-886B-C43662C6B702}" name="b" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -491,6 +491,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J138"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="23.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">

</xml_diff>